<commit_message>
Activa el refresco automático de tablas dinámicas en Mercadona-base.xlsx
Preparación única de la plantilla (hecha en Excel, no en código): las 7
tablas dinámicas comparten un único caché, y ahora tiene refreshOnLoad
activado ("Actualizar los datos al abrir el archivo"), por lo que
cualquier fichero que genere write-items-xlsx refrescará automáticamente
sus tablas y gráficos dinámicos al abrirse en Excel.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLvRfZo2QX1kb9xeztP44D
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" activeTab="7"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="6" r:id="rId1"/>
@@ -28,7 +28,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="55" r:id="rId9"/>
+    <pivotCache cacheId="8" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -181,31 +181,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
+  <dxfs count="24">
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     </dxf>
@@ -310,7 +286,6 @@
   </c:pivotSource>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -575,7 +550,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -677,7 +651,6 @@
   </c:pivotSource>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -957,7 +930,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1059,7 +1031,6 @@
   </c:pivotSource>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1379,7 +1350,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3199,7 +3169,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="dserrada@gmail.com" refreshedDate="46273.742382638891" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="3">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="dserrada@gmail.com" refreshedDate="46273.775013194441" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="3">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G1048576" sheet="Datos"/>
   </cacheSource>
@@ -3305,7 +3275,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending" defaultSubtotal="0">
@@ -3399,7 +3369,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0" defaultSubtotal="0"/>
@@ -3463,16 +3433,16 @@
     <dataField name="Suma de precio" fld="6" baseField="1" baseItem="10" numFmtId="164"/>
   </dataFields>
   <formats count="4">
-    <format dxfId="31">
+    <format dxfId="23">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="20">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3503,7 +3473,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
@@ -3577,16 +3547,16 @@
     <dataField name="Suma de unidades" fld="2" baseField="7" baseItem="0" numFmtId="1"/>
   </dataFields>
   <formats count="4">
-    <format dxfId="27">
+    <format dxfId="19">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="16">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3617,7 +3587,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A7:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" showAll="0" sortType="descending" defaultSubtotal="0">
@@ -3716,7 +3686,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending">
@@ -3816,7 +3786,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" multipleItemSelectionAllowed="1" showAll="0" sortType="descending">
@@ -3902,7 +3872,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="55" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A6:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisPage" showAll="0">

</xml_diff>

<commit_message>
Desactiva la retención de elementos obsoletos del campo id en Mercadona-base.xlsx
Las 6 tablas dinámicas que usan el campo "id" (todas salvo T_Precio)
retenían valores ya no presentes en los datos (Número de elementos a
retener = Automático), lo que dejaba un "4" fantasma en el selector de
filtro de la hoja Productos, sobrante de datos muy anteriores a las
2 filas de ejemplo actuales. Se pone missingItemsLimit="0" (Ninguno)
en esas 6 tablas para que el próximo refresco (el que ya se dispara
solo al abrir el fichero, por refreshOnLoad) purgue ese valor obsoleto.

Cambio aplicado editando directamente el XML del zip xlsx (verificado
que el resto de entradas del paquete queda byte a byte idéntico), ya
que no hay Excel disponible en este entorno para hacerlo desde la UI.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLvRfZo2QX1kb9xeztP44D
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -3275,7 +3275,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending" defaultSubtotal="0">
@@ -3473,7 +3473,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
@@ -3587,7 +3587,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A7:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" showAll="0" sortType="descending" defaultSubtotal="0">
@@ -3686,7 +3686,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending">
@@ -3786,7 +3786,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" multipleItemSelectionAllowed="1" showAll="0" sortType="descending">
@@ -3872,7 +3872,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A6:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisPage" showAll="0">

</xml_diff>

<commit_message>
Correcciones al excel base
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="6" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Mes" sheetId="10" r:id="rId5"/>
     <sheet name="Año" sheetId="12" r:id="rId6"/>
     <sheet name="Último" sheetId="13" r:id="rId7"/>
-    <sheet name="Evol" sheetId="14" r:id="rId8"/>
+    <sheet name="Subida" sheetId="14" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Datos!$A$1:$G$3</definedName>
@@ -28,7 +28,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId9"/>
+    <pivotCache cacheId="9" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,8 +38,76 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>dserrada@gmail.com</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>dserrada@gmail.com:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Para que en un futuro se pueda estimar que producto está a punto de acabarse. Es decir lleva más tiempo del normal sin comprarse</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>dserrada@gmail.com</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>dserrada@gmail.com:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Se promedia al mes porque hay productos de temporada</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="28">
   <si>
     <t>BARRA DE PAN</t>
   </si>
@@ -95,34 +163,34 @@
     <t>Cuenta de id</t>
   </si>
   <si>
-    <t>Promedio de unidades</t>
-  </si>
-  <si>
-    <t>Número de veces que se ha comprado un producto</t>
-  </si>
-  <si>
-    <t>Evolución Gasto al mes</t>
-  </si>
-  <si>
     <t>(Todas)</t>
-  </si>
-  <si>
-    <t>Promedio de unidades de un producto compradas al mes</t>
-  </si>
-  <si>
-    <t>Número de productos comprados al año</t>
   </si>
   <si>
     <t>Máx. de fecha</t>
   </si>
   <si>
-    <t>Ultima vez que compré un producto</t>
+    <t>Suma de unidades</t>
   </si>
   <si>
-    <t>Evolución del precio de un producto promediado al mes</t>
+    <t>Listado de productos comprados agrupados por el número de veces comprado. Incluye promedios sobre el producto</t>
   </si>
   <si>
-    <t>Suma de unidades</t>
+    <t>Número de productos comprados al mes. Con gráfica</t>
+  </si>
+  <si>
+    <t>Dinero gastado al mes. Con gráfica</t>
+  </si>
+  <si>
+    <t>Ultima vez que se compró un producto</t>
+  </si>
+  <si>
+    <t>Evolución del precio de un producto promediado al mes. En el selector se fija el producto y permite ver como ha evolucionado su precio con el tiempo</t>
+  </si>
+  <si>
+    <t>Promedio por mes de unidades de un producto. Con selectores para fijar el producto y el mes</t>
+  </si>
+  <si>
+    <t>Número de productos comprados al año. Especie de bolsa de la compara anual. Muestra cuanto se ha gastado en ese producto al año</t>
   </si>
 </sst>
 </file>
@@ -132,13 +200,26 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -161,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -174,38 +255,11 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     </dxf>
@@ -1026,11 +1080,12 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Mercadona-base.xlsx]Evol!TablaDinámica2</c:name>
+    <c:name>[Mercadona-base.xlsx]Subida!TablaDinámica2</c:name>
     <c:fmtId val="1"/>
   </c:pivotSource>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1157,7 +1212,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Evol!$B$6</c:f>
+              <c:f>Subida!$B$6</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1180,7 +1235,7 @@
           </c:marker>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Evol!$A$7:$A$11</c:f>
+              <c:f>Subida!$A$7:$A$11</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="2"/>
                 <c:lvl>
@@ -1204,7 +1259,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Evol!$B$7:$B$11</c:f>
+              <c:f>Subida!$B$7:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1350,6 +1405,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3169,7 +3225,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="dserrada@gmail.com" refreshedDate="46273.775013194441" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="3">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="dserrada@gmail.com" refreshedDate="46274.851091319448" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="3">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G1048576" sheet="Datos"/>
   </cacheSource>
@@ -3274,7 +3330,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending" defaultSubtotal="0">
@@ -3330,13 +3386,13 @@
   </rowFields>
   <rowItems count="4">
     <i>
+      <x/>
+    </i>
+    <i>
       <x v="1"/>
     </i>
     <i>
       <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -3367,7 +3423,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0" defaultSubtotal="0"/>
@@ -3431,16 +3487,16 @@
     <dataField name="Suma de precio" fld="6" baseField="1" baseItem="10" numFmtId="164"/>
   </dataFields>
   <formats count="4">
-    <format dxfId="23">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="12">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3471,7 +3527,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
@@ -3544,16 +3600,16 @@
     <dataField name="Suma de unidades" fld="2" baseField="7" baseItem="0" numFmtId="1"/>
   </dataFields>
   <formats count="4">
-    <format dxfId="19">
+    <format dxfId="11">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="8">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3584,7 +3640,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A7:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" showAll="0" sortType="descending" defaultSubtotal="0">
@@ -3640,13 +3696,13 @@
   </rowFields>
   <rowItems count="4">
     <i>
-      <x v="2"/>
-    </i>
-    <i>
       <x v="1"/>
     </i>
     <i>
-      <x v="3"/>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
     </i>
     <i t="grand">
       <x/>
@@ -3659,7 +3715,7 @@
     <pageField fld="1" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="Promedio de unidades" fld="2" subtotal="average" baseField="0" baseItem="9" numFmtId="1"/>
+    <dataField name="Suma de unidades" fld="2" baseField="0" baseItem="1" numFmtId="1"/>
   </dataFields>
   <chartFormats count="1">
     <chartFormat chart="0" format="4" series="1">
@@ -3682,8 +3738,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A4:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A4:C10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending">
       <items count="4">
@@ -3696,13 +3752,13 @@
         <pivotArea dataOnly="0" outline="0" fieldPosition="0">
           <references count="1">
             <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
+              <x v="1"/>
             </reference>
           </references>
         </pivotArea>
       </autoSortScope>
     </pivotField>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0">
       <items count="15">
         <item x="0"/>
         <item x="1"/>
@@ -3725,7 +3781,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -3734,42 +3790,44 @@
       </items>
     </pivotField>
   </pivotFields>
-  <rowFields count="3">
+  <rowFields count="2">
     <field x="7"/>
-    <field x="1"/>
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
+  <rowItems count="6">
     <i>
       <x/>
     </i>
     <i r="1">
-      <x/>
-    </i>
-    <i r="2">
-      <x v="3"/>
+      <x v="2"/>
     </i>
     <i>
       <x v="1"/>
     </i>
     <i r="1">
-      <x v="6"/>
+      <x v="1"/>
     </i>
-    <i r="2">
-      <x v="2"/>
-    </i>
-    <i r="2">
-      <x v="1"/>
+    <i r="1">
+      <x/>
     </i>
     <i t="grand">
       <x/>
     </i>
   </rowItems>
-  <colItems count="1">
-    <i/>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
   </colItems>
-  <dataFields count="1">
+  <dataFields count="2">
     <dataField name="Cuenta de id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Suma de precio" fld="6" baseField="0" baseItem="1"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -3781,7 +3839,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" multipleItemSelectionAllowed="1" showAll="0" sortType="descending">
@@ -3838,13 +3896,13 @@
   </rowFields>
   <rowItems count="4">
     <i>
+      <x/>
+    </i>
+    <i>
       <x v="1"/>
     </i>
     <i>
       <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -3866,7 +3924,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="8" missingItemsLimit="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A6:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisPage" showAll="0">
@@ -4228,10 +4286,10 @@
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -4310,7 +4368,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -6031,7 +6089,7 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B1"/>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -19797,7 +19855,7 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B1"/>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -19805,7 +19863,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -19813,7 +19871,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C4"/>
     </row>
@@ -33564,12 +33622,12 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -33577,7 +33635,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -33585,7 +33643,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -33615,7 +33673,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="7">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -33625,16 +33683,17 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
     <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -33644,61 +33703,62 @@
       <c r="B4" t="s">
         <v>17</v>
       </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>3</v>
+      <c r="A7" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
+      <c r="A8" s="5" t="s">
+        <v>1</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="4">
+        <v>1</v>
+      </c>
+      <c r="C8" s="4">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B9" s="4">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="4">
-        <v>2</v>
+      <c r="C10" s="4">
+        <v>3.98</v>
       </c>
     </row>
   </sheetData>
@@ -33707,7 +33767,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -33717,7 +33777,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -33725,7 +33785,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -33761,11 +33821,12 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -33776,7 +33837,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -33784,7 +33845,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -33832,5 +33893,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Añade hoja Evolucion-N a Mercadona-base.xlsx y repara estilo de porcentaje perdido
Al guardar la plantilla desde Excel (para añadir la hoja, gráfico y tabla
dinámica de Evolucion-N), Excel eliminó por "no usado" el estilo de
porcentaje (cellXfs índice 8, numFmtId 10) que XlsxDatosWriter necesita
para la hoja MiInflación, ya que ninguna celda de la propia plantilla lo
referencia directamente. Esto hacía que el xlsx generado quedara con una
referencia de estilo inválida y Excel lo marcara como dañado al abrirlo.
Se restaura esa entrada de estilo conservando el resto de cambios de la
plantilla.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qDQuYQVFErjUJZQGtd4PP
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="6" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="Mes" sheetId="10" r:id="rId6"/>
     <sheet name="Año" sheetId="12" r:id="rId7"/>
     <sheet name="Último" sheetId="13" r:id="rId8"/>
-    <sheet name="Subida" sheetId="14" r:id="rId9"/>
+    <sheet name="Evolucion-€" sheetId="14" r:id="rId9"/>
+    <sheet name="Evolucion-N" sheetId="17" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Datos!$A$1:$G$3</definedName>
@@ -29,7 +30,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId10"/>
+    <pivotCache cacheId="4" r:id="rId11"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -108,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="36">
   <si>
     <t>BARRA DE PAN</t>
   </si>
@@ -213,6 +214,9 @@
   </si>
   <si>
     <t>Productos coincidentes</t>
+  </si>
+  <si>
+    <t>Evolución de la cantidad de productos comprados en un año. En el selector se fija el producto y permite ver como ha evolucionadoel número de productos comprados</t>
   </si>
 </sst>
 </file>
@@ -1103,11 +1107,12 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Mercadona-base.xlsx]Subida!TablaDinámica2</c:name>
+    <c:name>[Mercadona-base.xlsx]Evolucion-€!TablaDinámica2</c:name>
     <c:fmtId val="1"/>
   </c:pivotSource>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1234,7 +1239,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Subida!$B$6</c:f>
+              <c:f>'Evolucion-€'!$B$6</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1257,7 +1262,7 @@
           </c:marker>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Subida!$A$7:$A$11</c:f>
+              <c:f>'Evolucion-€'!$A$7:$A$11</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="2"/>
                 <c:lvl>
@@ -1281,7 +1286,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Subida!$B$7:$B$11</c:f>
+              <c:f>'Evolucion-€'!$B$7:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1427,6 +1432,368 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Mercadona-base.xlsx]Evolucion-N!TablaDinámica1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="28575" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:ln w="28575" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Evolucion-N'!$B$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Evolucion-N'!$A$7:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>&lt;16/06/2023</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Evolucion-N'!$B$7:$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5B05-4E5C-82B9-86F8C05DAFB5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="557855232"/>
+        <c:axId val="557857312"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="557855232"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="557857312"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="557857312"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="557855232"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1590,6 +1957,46 @@
 </file>
 
 <file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -3138,6 +3545,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -3245,8 +4168,43 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>619125</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="dserrada@gmail.com" refreshedDate="46275.604974768517" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="3">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="dserrada@gmail.com" refreshedDate="46277.655617592594" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="3">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G1048576" sheet="Datos"/>
   </cacheSource>
@@ -4038,6 +4996,75 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="A6:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="8">
+    <pivotField axis="axisPage" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="0" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Suma de unidades" fld="2" baseField="7" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -4377,6 +5404,64 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D558"/>

</xml_diff>

<commit_message>
Añade la hoja Interanual (mismo mes, distintos años) a la plantilla xlsx
Nueva hoja "Interanual" en Mercadona-base.xlsx, antes de "T_Precio":
tabla dinámica sobre la caché común con el gasto por mes (filas) y año
(columnas) y, debajo, el % de variación de cada mes frente al mismo mes
del año anterior, en rojo/verde.

La variación se calcula con fórmulas que leen la tabla por posición en
vez de con "% de diferencia respecto al anterior" de la tabla dinámica,
porque LibreOffice no lo calcula sobre un campo agrupado y no se podía
verificar fuera de Excel. El total anual se sustituye por un "Total
(meses comparables)" que solo suma los meses con gasto en los dos años,
para que el primer y el último año, incompletos, no distorsionen la
comparación.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Productos" sheetId="7" r:id="rId2"/>
     <sheet name="Pareto" sheetId="18" r:id="rId15"/>
     <sheet name="MiInflación" sheetId="16" r:id="rId3"/>
+    <sheet name="Interanual" sheetId="19" r:id="rId16"/>
     <sheet name="T_Precio" sheetId="8" r:id="rId4"/>
     <sheet name="T_Cantidad" sheetId="15" r:id="rId5"/>
     <sheet name="Mes" sheetId="10" r:id="rId6"/>
@@ -227,7 +228,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,6 +248,30 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -293,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -314,11 +339,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="21">
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     </dxf>
@@ -399,6 +428,16 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4466,6 +4505,76 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámicaInteranual" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
+      <items count="14">
+        <item x="0" h="1"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisCol" showAll="0" defaultSubtotal="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x v="6"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="7"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Gasto" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
@@ -21730,6 +21839,924 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P41"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="16" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interanual: el mismo mes en distintos años</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compara cada mes con el mismo mes de otros años, separando la estacionalidad (p. ej. diciembre siempre es más caro) de la tendencia real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ojo: el primer y el último año de la serie (y el mes en curso) suelen estar incompletos; por eso el total interanual solo compara los meses con datos en los dos años.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gasto por mes y año</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Etiquetas de fila</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% de variación frente al mismo mes del año anterior (rojo: gastas más; verde: gastas menos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mes</t>
+        </is>
+      </c>
+      <c r="B25" s="15">
+        <f>IF(OR(B$6="",ISERROR(VALUE(B$6))),"",B$6)</f>
+      </c>
+      <c r="C25" s="15">
+        <f>IF(OR(C$6="",ISERROR(VALUE(C$6))),"",C$6)</f>
+      </c>
+      <c r="D25" s="15">
+        <f>IF(OR(D$6="",ISERROR(VALUE(D$6))),"",D$6)</f>
+      </c>
+      <c r="E25" s="15">
+        <f>IF(OR(E$6="",ISERROR(VALUE(E$6))),"",E$6)</f>
+      </c>
+      <c r="F25" s="15">
+        <f>IF(OR(F$6="",ISERROR(VALUE(F$6))),"",F$6)</f>
+      </c>
+      <c r="G25" s="15">
+        <f>IF(OR(G$6="",ISERROR(VALUE(G$6))),"",G$6)</f>
+      </c>
+      <c r="H25" s="15">
+        <f>IF(OR(H$6="",ISERROR(VALUE(H$6))),"",H$6)</f>
+      </c>
+      <c r="I25" s="15">
+        <f>IF(OR(I$6="",ISERROR(VALUE(I$6))),"",I$6)</f>
+      </c>
+      <c r="J25" s="15">
+        <f>IF(OR(J$6="",ISERROR(VALUE(J$6))),"",J$6)</f>
+      </c>
+      <c r="K25" s="15">
+        <f>IF(OR(K$6="",ISERROR(VALUE(K$6))),"",K$6)</f>
+      </c>
+      <c r="L25" s="15">
+        <f>IF(OR(L$6="",ISERROR(VALUE(L$6))),"",L$6)</f>
+      </c>
+      <c r="M25" s="15">
+        <f>IF(OR(M$6="",ISERROR(VALUE(M$6))),"",M$6)</f>
+      </c>
+      <c r="N25" s="15">
+        <f>IF(OR(N$6="",ISERROR(VALUE(N$6))),"",N$6)</f>
+      </c>
+      <c r="O25" s="15">
+        <f>IF(OR(O$6="",ISERROR(VALUE(O$6))),"",O$6)</f>
+      </c>
+      <c r="P25" s="15">
+        <f>IF(OR(P$6="",ISERROR(VALUE(P$6))),"",P$6)</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <f>IF(OR(A7="",A8=""),"",A7)</f>
+      </c>
+      <c r="B26" s="17">
+        <f>IF(OR(B$25="",$A26="",NOT(ISNUMBER(B7)),NOT(ISNUMBER(A7)),N(A7)=0),"",B7/A7-1)</f>
+      </c>
+      <c r="C26" s="17">
+        <f>IF(OR(C$25="",$A26="",NOT(ISNUMBER(C7)),NOT(ISNUMBER(B7)),N(B7)=0),"",C7/B7-1)</f>
+      </c>
+      <c r="D26" s="17">
+        <f>IF(OR(D$25="",$A26="",NOT(ISNUMBER(D7)),NOT(ISNUMBER(C7)),N(C7)=0),"",D7/C7-1)</f>
+      </c>
+      <c r="E26" s="17">
+        <f>IF(OR(E$25="",$A26="",NOT(ISNUMBER(E7)),NOT(ISNUMBER(D7)),N(D7)=0),"",E7/D7-1)</f>
+      </c>
+      <c r="F26" s="17">
+        <f>IF(OR(F$25="",$A26="",NOT(ISNUMBER(F7)),NOT(ISNUMBER(E7)),N(E7)=0),"",F7/E7-1)</f>
+      </c>
+      <c r="G26" s="17">
+        <f>IF(OR(G$25="",$A26="",NOT(ISNUMBER(G7)),NOT(ISNUMBER(F7)),N(F7)=0),"",G7/F7-1)</f>
+      </c>
+      <c r="H26" s="17">
+        <f>IF(OR(H$25="",$A26="",NOT(ISNUMBER(H7)),NOT(ISNUMBER(G7)),N(G7)=0),"",H7/G7-1)</f>
+      </c>
+      <c r="I26" s="17">
+        <f>IF(OR(I$25="",$A26="",NOT(ISNUMBER(I7)),NOT(ISNUMBER(H7)),N(H7)=0),"",I7/H7-1)</f>
+      </c>
+      <c r="J26" s="17">
+        <f>IF(OR(J$25="",$A26="",NOT(ISNUMBER(J7)),NOT(ISNUMBER(I7)),N(I7)=0),"",J7/I7-1)</f>
+      </c>
+      <c r="K26" s="17">
+        <f>IF(OR(K$25="",$A26="",NOT(ISNUMBER(K7)),NOT(ISNUMBER(J7)),N(J7)=0),"",K7/J7-1)</f>
+      </c>
+      <c r="L26" s="17">
+        <f>IF(OR(L$25="",$A26="",NOT(ISNUMBER(L7)),NOT(ISNUMBER(K7)),N(K7)=0),"",L7/K7-1)</f>
+      </c>
+      <c r="M26" s="17">
+        <f>IF(OR(M$25="",$A26="",NOT(ISNUMBER(M7)),NOT(ISNUMBER(L7)),N(L7)=0),"",M7/L7-1)</f>
+      </c>
+      <c r="N26" s="17">
+        <f>IF(OR(N$25="",$A26="",NOT(ISNUMBER(N7)),NOT(ISNUMBER(M7)),N(M7)=0),"",N7/M7-1)</f>
+      </c>
+      <c r="O26" s="17">
+        <f>IF(OR(O$25="",$A26="",NOT(ISNUMBER(O7)),NOT(ISNUMBER(N7)),N(N7)=0),"",O7/N7-1)</f>
+      </c>
+      <c r="P26" s="17">
+        <f>IF(OR(P$25="",$A26="",NOT(ISNUMBER(P7)),NOT(ISNUMBER(O7)),N(O7)=0),"",P7/O7-1)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <f>IF(OR(A8="",A9=""),"",A8)</f>
+      </c>
+      <c r="B27" s="17">
+        <f>IF(OR(B$25="",$A27="",NOT(ISNUMBER(B8)),NOT(ISNUMBER(A8)),N(A8)=0),"",B8/A8-1)</f>
+      </c>
+      <c r="C27" s="17">
+        <f>IF(OR(C$25="",$A27="",NOT(ISNUMBER(C8)),NOT(ISNUMBER(B8)),N(B8)=0),"",C8/B8-1)</f>
+      </c>
+      <c r="D27" s="17">
+        <f>IF(OR(D$25="",$A27="",NOT(ISNUMBER(D8)),NOT(ISNUMBER(C8)),N(C8)=0),"",D8/C8-1)</f>
+      </c>
+      <c r="E27" s="17">
+        <f>IF(OR(E$25="",$A27="",NOT(ISNUMBER(E8)),NOT(ISNUMBER(D8)),N(D8)=0),"",E8/D8-1)</f>
+      </c>
+      <c r="F27" s="17">
+        <f>IF(OR(F$25="",$A27="",NOT(ISNUMBER(F8)),NOT(ISNUMBER(E8)),N(E8)=0),"",F8/E8-1)</f>
+      </c>
+      <c r="G27" s="17">
+        <f>IF(OR(G$25="",$A27="",NOT(ISNUMBER(G8)),NOT(ISNUMBER(F8)),N(F8)=0),"",G8/F8-1)</f>
+      </c>
+      <c r="H27" s="17">
+        <f>IF(OR(H$25="",$A27="",NOT(ISNUMBER(H8)),NOT(ISNUMBER(G8)),N(G8)=0),"",H8/G8-1)</f>
+      </c>
+      <c r="I27" s="17">
+        <f>IF(OR(I$25="",$A27="",NOT(ISNUMBER(I8)),NOT(ISNUMBER(H8)),N(H8)=0),"",I8/H8-1)</f>
+      </c>
+      <c r="J27" s="17">
+        <f>IF(OR(J$25="",$A27="",NOT(ISNUMBER(J8)),NOT(ISNUMBER(I8)),N(I8)=0),"",J8/I8-1)</f>
+      </c>
+      <c r="K27" s="17">
+        <f>IF(OR(K$25="",$A27="",NOT(ISNUMBER(K8)),NOT(ISNUMBER(J8)),N(J8)=0),"",K8/J8-1)</f>
+      </c>
+      <c r="L27" s="17">
+        <f>IF(OR(L$25="",$A27="",NOT(ISNUMBER(L8)),NOT(ISNUMBER(K8)),N(K8)=0),"",L8/K8-1)</f>
+      </c>
+      <c r="M27" s="17">
+        <f>IF(OR(M$25="",$A27="",NOT(ISNUMBER(M8)),NOT(ISNUMBER(L8)),N(L8)=0),"",M8/L8-1)</f>
+      </c>
+      <c r="N27" s="17">
+        <f>IF(OR(N$25="",$A27="",NOT(ISNUMBER(N8)),NOT(ISNUMBER(M8)),N(M8)=0),"",N8/M8-1)</f>
+      </c>
+      <c r="O27" s="17">
+        <f>IF(OR(O$25="",$A27="",NOT(ISNUMBER(O8)),NOT(ISNUMBER(N8)),N(N8)=0),"",O8/N8-1)</f>
+      </c>
+      <c r="P27" s="17">
+        <f>IF(OR(P$25="",$A27="",NOT(ISNUMBER(P8)),NOT(ISNUMBER(O8)),N(O8)=0),"",P8/O8-1)</f>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <f>IF(OR(A9="",A10=""),"",A9)</f>
+      </c>
+      <c r="B28" s="17">
+        <f>IF(OR(B$25="",$A28="",NOT(ISNUMBER(B9)),NOT(ISNUMBER(A9)),N(A9)=0),"",B9/A9-1)</f>
+      </c>
+      <c r="C28" s="17">
+        <f>IF(OR(C$25="",$A28="",NOT(ISNUMBER(C9)),NOT(ISNUMBER(B9)),N(B9)=0),"",C9/B9-1)</f>
+      </c>
+      <c r="D28" s="17">
+        <f>IF(OR(D$25="",$A28="",NOT(ISNUMBER(D9)),NOT(ISNUMBER(C9)),N(C9)=0),"",D9/C9-1)</f>
+      </c>
+      <c r="E28" s="17">
+        <f>IF(OR(E$25="",$A28="",NOT(ISNUMBER(E9)),NOT(ISNUMBER(D9)),N(D9)=0),"",E9/D9-1)</f>
+      </c>
+      <c r="F28" s="17">
+        <f>IF(OR(F$25="",$A28="",NOT(ISNUMBER(F9)),NOT(ISNUMBER(E9)),N(E9)=0),"",F9/E9-1)</f>
+      </c>
+      <c r="G28" s="17">
+        <f>IF(OR(G$25="",$A28="",NOT(ISNUMBER(G9)),NOT(ISNUMBER(F9)),N(F9)=0),"",G9/F9-1)</f>
+      </c>
+      <c r="H28" s="17">
+        <f>IF(OR(H$25="",$A28="",NOT(ISNUMBER(H9)),NOT(ISNUMBER(G9)),N(G9)=0),"",H9/G9-1)</f>
+      </c>
+      <c r="I28" s="17">
+        <f>IF(OR(I$25="",$A28="",NOT(ISNUMBER(I9)),NOT(ISNUMBER(H9)),N(H9)=0),"",I9/H9-1)</f>
+      </c>
+      <c r="J28" s="17">
+        <f>IF(OR(J$25="",$A28="",NOT(ISNUMBER(J9)),NOT(ISNUMBER(I9)),N(I9)=0),"",J9/I9-1)</f>
+      </c>
+      <c r="K28" s="17">
+        <f>IF(OR(K$25="",$A28="",NOT(ISNUMBER(K9)),NOT(ISNUMBER(J9)),N(J9)=0),"",K9/J9-1)</f>
+      </c>
+      <c r="L28" s="17">
+        <f>IF(OR(L$25="",$A28="",NOT(ISNUMBER(L9)),NOT(ISNUMBER(K9)),N(K9)=0),"",L9/K9-1)</f>
+      </c>
+      <c r="M28" s="17">
+        <f>IF(OR(M$25="",$A28="",NOT(ISNUMBER(M9)),NOT(ISNUMBER(L9)),N(L9)=0),"",M9/L9-1)</f>
+      </c>
+      <c r="N28" s="17">
+        <f>IF(OR(N$25="",$A28="",NOT(ISNUMBER(N9)),NOT(ISNUMBER(M9)),N(M9)=0),"",N9/M9-1)</f>
+      </c>
+      <c r="O28" s="17">
+        <f>IF(OR(O$25="",$A28="",NOT(ISNUMBER(O9)),NOT(ISNUMBER(N9)),N(N9)=0),"",O9/N9-1)</f>
+      </c>
+      <c r="P28" s="17">
+        <f>IF(OR(P$25="",$A28="",NOT(ISNUMBER(P9)),NOT(ISNUMBER(O9)),N(O9)=0),"",P9/O9-1)</f>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <f>IF(OR(A10="",A11=""),"",A10)</f>
+      </c>
+      <c r="B29" s="17">
+        <f>IF(OR(B$25="",$A29="",NOT(ISNUMBER(B10)),NOT(ISNUMBER(A10)),N(A10)=0),"",B10/A10-1)</f>
+      </c>
+      <c r="C29" s="17">
+        <f>IF(OR(C$25="",$A29="",NOT(ISNUMBER(C10)),NOT(ISNUMBER(B10)),N(B10)=0),"",C10/B10-1)</f>
+      </c>
+      <c r="D29" s="17">
+        <f>IF(OR(D$25="",$A29="",NOT(ISNUMBER(D10)),NOT(ISNUMBER(C10)),N(C10)=0),"",D10/C10-1)</f>
+      </c>
+      <c r="E29" s="17">
+        <f>IF(OR(E$25="",$A29="",NOT(ISNUMBER(E10)),NOT(ISNUMBER(D10)),N(D10)=0),"",E10/D10-1)</f>
+      </c>
+      <c r="F29" s="17">
+        <f>IF(OR(F$25="",$A29="",NOT(ISNUMBER(F10)),NOT(ISNUMBER(E10)),N(E10)=0),"",F10/E10-1)</f>
+      </c>
+      <c r="G29" s="17">
+        <f>IF(OR(G$25="",$A29="",NOT(ISNUMBER(G10)),NOT(ISNUMBER(F10)),N(F10)=0),"",G10/F10-1)</f>
+      </c>
+      <c r="H29" s="17">
+        <f>IF(OR(H$25="",$A29="",NOT(ISNUMBER(H10)),NOT(ISNUMBER(G10)),N(G10)=0),"",H10/G10-1)</f>
+      </c>
+      <c r="I29" s="17">
+        <f>IF(OR(I$25="",$A29="",NOT(ISNUMBER(I10)),NOT(ISNUMBER(H10)),N(H10)=0),"",I10/H10-1)</f>
+      </c>
+      <c r="J29" s="17">
+        <f>IF(OR(J$25="",$A29="",NOT(ISNUMBER(J10)),NOT(ISNUMBER(I10)),N(I10)=0),"",J10/I10-1)</f>
+      </c>
+      <c r="K29" s="17">
+        <f>IF(OR(K$25="",$A29="",NOT(ISNUMBER(K10)),NOT(ISNUMBER(J10)),N(J10)=0),"",K10/J10-1)</f>
+      </c>
+      <c r="L29" s="17">
+        <f>IF(OR(L$25="",$A29="",NOT(ISNUMBER(L10)),NOT(ISNUMBER(K10)),N(K10)=0),"",L10/K10-1)</f>
+      </c>
+      <c r="M29" s="17">
+        <f>IF(OR(M$25="",$A29="",NOT(ISNUMBER(M10)),NOT(ISNUMBER(L10)),N(L10)=0),"",M10/L10-1)</f>
+      </c>
+      <c r="N29" s="17">
+        <f>IF(OR(N$25="",$A29="",NOT(ISNUMBER(N10)),NOT(ISNUMBER(M10)),N(M10)=0),"",N10/M10-1)</f>
+      </c>
+      <c r="O29" s="17">
+        <f>IF(OR(O$25="",$A29="",NOT(ISNUMBER(O10)),NOT(ISNUMBER(N10)),N(N10)=0),"",O10/N10-1)</f>
+      </c>
+      <c r="P29" s="17">
+        <f>IF(OR(P$25="",$A29="",NOT(ISNUMBER(P10)),NOT(ISNUMBER(O10)),N(O10)=0),"",P10/O10-1)</f>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <f>IF(OR(A11="",A12=""),"",A11)</f>
+      </c>
+      <c r="B30" s="17">
+        <f>IF(OR(B$25="",$A30="",NOT(ISNUMBER(B11)),NOT(ISNUMBER(A11)),N(A11)=0),"",B11/A11-1)</f>
+      </c>
+      <c r="C30" s="17">
+        <f>IF(OR(C$25="",$A30="",NOT(ISNUMBER(C11)),NOT(ISNUMBER(B11)),N(B11)=0),"",C11/B11-1)</f>
+      </c>
+      <c r="D30" s="17">
+        <f>IF(OR(D$25="",$A30="",NOT(ISNUMBER(D11)),NOT(ISNUMBER(C11)),N(C11)=0),"",D11/C11-1)</f>
+      </c>
+      <c r="E30" s="17">
+        <f>IF(OR(E$25="",$A30="",NOT(ISNUMBER(E11)),NOT(ISNUMBER(D11)),N(D11)=0),"",E11/D11-1)</f>
+      </c>
+      <c r="F30" s="17">
+        <f>IF(OR(F$25="",$A30="",NOT(ISNUMBER(F11)),NOT(ISNUMBER(E11)),N(E11)=0),"",F11/E11-1)</f>
+      </c>
+      <c r="G30" s="17">
+        <f>IF(OR(G$25="",$A30="",NOT(ISNUMBER(G11)),NOT(ISNUMBER(F11)),N(F11)=0),"",G11/F11-1)</f>
+      </c>
+      <c r="H30" s="17">
+        <f>IF(OR(H$25="",$A30="",NOT(ISNUMBER(H11)),NOT(ISNUMBER(G11)),N(G11)=0),"",H11/G11-1)</f>
+      </c>
+      <c r="I30" s="17">
+        <f>IF(OR(I$25="",$A30="",NOT(ISNUMBER(I11)),NOT(ISNUMBER(H11)),N(H11)=0),"",I11/H11-1)</f>
+      </c>
+      <c r="J30" s="17">
+        <f>IF(OR(J$25="",$A30="",NOT(ISNUMBER(J11)),NOT(ISNUMBER(I11)),N(I11)=0),"",J11/I11-1)</f>
+      </c>
+      <c r="K30" s="17">
+        <f>IF(OR(K$25="",$A30="",NOT(ISNUMBER(K11)),NOT(ISNUMBER(J11)),N(J11)=0),"",K11/J11-1)</f>
+      </c>
+      <c r="L30" s="17">
+        <f>IF(OR(L$25="",$A30="",NOT(ISNUMBER(L11)),NOT(ISNUMBER(K11)),N(K11)=0),"",L11/K11-1)</f>
+      </c>
+      <c r="M30" s="17">
+        <f>IF(OR(M$25="",$A30="",NOT(ISNUMBER(M11)),NOT(ISNUMBER(L11)),N(L11)=0),"",M11/L11-1)</f>
+      </c>
+      <c r="N30" s="17">
+        <f>IF(OR(N$25="",$A30="",NOT(ISNUMBER(N11)),NOT(ISNUMBER(M11)),N(M11)=0),"",N11/M11-1)</f>
+      </c>
+      <c r="O30" s="17">
+        <f>IF(OR(O$25="",$A30="",NOT(ISNUMBER(O11)),NOT(ISNUMBER(N11)),N(N11)=0),"",O11/N11-1)</f>
+      </c>
+      <c r="P30" s="17">
+        <f>IF(OR(P$25="",$A30="",NOT(ISNUMBER(P11)),NOT(ISNUMBER(O11)),N(O11)=0),"",P11/O11-1)</f>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <f>IF(OR(A12="",A13=""),"",A12)</f>
+      </c>
+      <c r="B31" s="17">
+        <f>IF(OR(B$25="",$A31="",NOT(ISNUMBER(B12)),NOT(ISNUMBER(A12)),N(A12)=0),"",B12/A12-1)</f>
+      </c>
+      <c r="C31" s="17">
+        <f>IF(OR(C$25="",$A31="",NOT(ISNUMBER(C12)),NOT(ISNUMBER(B12)),N(B12)=0),"",C12/B12-1)</f>
+      </c>
+      <c r="D31" s="17">
+        <f>IF(OR(D$25="",$A31="",NOT(ISNUMBER(D12)),NOT(ISNUMBER(C12)),N(C12)=0),"",D12/C12-1)</f>
+      </c>
+      <c r="E31" s="17">
+        <f>IF(OR(E$25="",$A31="",NOT(ISNUMBER(E12)),NOT(ISNUMBER(D12)),N(D12)=0),"",E12/D12-1)</f>
+      </c>
+      <c r="F31" s="17">
+        <f>IF(OR(F$25="",$A31="",NOT(ISNUMBER(F12)),NOT(ISNUMBER(E12)),N(E12)=0),"",F12/E12-1)</f>
+      </c>
+      <c r="G31" s="17">
+        <f>IF(OR(G$25="",$A31="",NOT(ISNUMBER(G12)),NOT(ISNUMBER(F12)),N(F12)=0),"",G12/F12-1)</f>
+      </c>
+      <c r="H31" s="17">
+        <f>IF(OR(H$25="",$A31="",NOT(ISNUMBER(H12)),NOT(ISNUMBER(G12)),N(G12)=0),"",H12/G12-1)</f>
+      </c>
+      <c r="I31" s="17">
+        <f>IF(OR(I$25="",$A31="",NOT(ISNUMBER(I12)),NOT(ISNUMBER(H12)),N(H12)=0),"",I12/H12-1)</f>
+      </c>
+      <c r="J31" s="17">
+        <f>IF(OR(J$25="",$A31="",NOT(ISNUMBER(J12)),NOT(ISNUMBER(I12)),N(I12)=0),"",J12/I12-1)</f>
+      </c>
+      <c r="K31" s="17">
+        <f>IF(OR(K$25="",$A31="",NOT(ISNUMBER(K12)),NOT(ISNUMBER(J12)),N(J12)=0),"",K12/J12-1)</f>
+      </c>
+      <c r="L31" s="17">
+        <f>IF(OR(L$25="",$A31="",NOT(ISNUMBER(L12)),NOT(ISNUMBER(K12)),N(K12)=0),"",L12/K12-1)</f>
+      </c>
+      <c r="M31" s="17">
+        <f>IF(OR(M$25="",$A31="",NOT(ISNUMBER(M12)),NOT(ISNUMBER(L12)),N(L12)=0),"",M12/L12-1)</f>
+      </c>
+      <c r="N31" s="17">
+        <f>IF(OR(N$25="",$A31="",NOT(ISNUMBER(N12)),NOT(ISNUMBER(M12)),N(M12)=0),"",N12/M12-1)</f>
+      </c>
+      <c r="O31" s="17">
+        <f>IF(OR(O$25="",$A31="",NOT(ISNUMBER(O12)),NOT(ISNUMBER(N12)),N(N12)=0),"",O12/N12-1)</f>
+      </c>
+      <c r="P31" s="17">
+        <f>IF(OR(P$25="",$A31="",NOT(ISNUMBER(P12)),NOT(ISNUMBER(O12)),N(O12)=0),"",P12/O12-1)</f>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <f>IF(OR(A13="",A14=""),"",A13)</f>
+      </c>
+      <c r="B32" s="17">
+        <f>IF(OR(B$25="",$A32="",NOT(ISNUMBER(B13)),NOT(ISNUMBER(A13)),N(A13)=0),"",B13/A13-1)</f>
+      </c>
+      <c r="C32" s="17">
+        <f>IF(OR(C$25="",$A32="",NOT(ISNUMBER(C13)),NOT(ISNUMBER(B13)),N(B13)=0),"",C13/B13-1)</f>
+      </c>
+      <c r="D32" s="17">
+        <f>IF(OR(D$25="",$A32="",NOT(ISNUMBER(D13)),NOT(ISNUMBER(C13)),N(C13)=0),"",D13/C13-1)</f>
+      </c>
+      <c r="E32" s="17">
+        <f>IF(OR(E$25="",$A32="",NOT(ISNUMBER(E13)),NOT(ISNUMBER(D13)),N(D13)=0),"",E13/D13-1)</f>
+      </c>
+      <c r="F32" s="17">
+        <f>IF(OR(F$25="",$A32="",NOT(ISNUMBER(F13)),NOT(ISNUMBER(E13)),N(E13)=0),"",F13/E13-1)</f>
+      </c>
+      <c r="G32" s="17">
+        <f>IF(OR(G$25="",$A32="",NOT(ISNUMBER(G13)),NOT(ISNUMBER(F13)),N(F13)=0),"",G13/F13-1)</f>
+      </c>
+      <c r="H32" s="17">
+        <f>IF(OR(H$25="",$A32="",NOT(ISNUMBER(H13)),NOT(ISNUMBER(G13)),N(G13)=0),"",H13/G13-1)</f>
+      </c>
+      <c r="I32" s="17">
+        <f>IF(OR(I$25="",$A32="",NOT(ISNUMBER(I13)),NOT(ISNUMBER(H13)),N(H13)=0),"",I13/H13-1)</f>
+      </c>
+      <c r="J32" s="17">
+        <f>IF(OR(J$25="",$A32="",NOT(ISNUMBER(J13)),NOT(ISNUMBER(I13)),N(I13)=0),"",J13/I13-1)</f>
+      </c>
+      <c r="K32" s="17">
+        <f>IF(OR(K$25="",$A32="",NOT(ISNUMBER(K13)),NOT(ISNUMBER(J13)),N(J13)=0),"",K13/J13-1)</f>
+      </c>
+      <c r="L32" s="17">
+        <f>IF(OR(L$25="",$A32="",NOT(ISNUMBER(L13)),NOT(ISNUMBER(K13)),N(K13)=0),"",L13/K13-1)</f>
+      </c>
+      <c r="M32" s="17">
+        <f>IF(OR(M$25="",$A32="",NOT(ISNUMBER(M13)),NOT(ISNUMBER(L13)),N(L13)=0),"",M13/L13-1)</f>
+      </c>
+      <c r="N32" s="17">
+        <f>IF(OR(N$25="",$A32="",NOT(ISNUMBER(N13)),NOT(ISNUMBER(M13)),N(M13)=0),"",N13/M13-1)</f>
+      </c>
+      <c r="O32" s="17">
+        <f>IF(OR(O$25="",$A32="",NOT(ISNUMBER(O13)),NOT(ISNUMBER(N13)),N(N13)=0),"",O13/N13-1)</f>
+      </c>
+      <c r="P32" s="17">
+        <f>IF(OR(P$25="",$A32="",NOT(ISNUMBER(P13)),NOT(ISNUMBER(O13)),N(O13)=0),"",P13/O13-1)</f>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <f>IF(OR(A14="",A15=""),"",A14)</f>
+      </c>
+      <c r="B33" s="17">
+        <f>IF(OR(B$25="",$A33="",NOT(ISNUMBER(B14)),NOT(ISNUMBER(A14)),N(A14)=0),"",B14/A14-1)</f>
+      </c>
+      <c r="C33" s="17">
+        <f>IF(OR(C$25="",$A33="",NOT(ISNUMBER(C14)),NOT(ISNUMBER(B14)),N(B14)=0),"",C14/B14-1)</f>
+      </c>
+      <c r="D33" s="17">
+        <f>IF(OR(D$25="",$A33="",NOT(ISNUMBER(D14)),NOT(ISNUMBER(C14)),N(C14)=0),"",D14/C14-1)</f>
+      </c>
+      <c r="E33" s="17">
+        <f>IF(OR(E$25="",$A33="",NOT(ISNUMBER(E14)),NOT(ISNUMBER(D14)),N(D14)=0),"",E14/D14-1)</f>
+      </c>
+      <c r="F33" s="17">
+        <f>IF(OR(F$25="",$A33="",NOT(ISNUMBER(F14)),NOT(ISNUMBER(E14)),N(E14)=0),"",F14/E14-1)</f>
+      </c>
+      <c r="G33" s="17">
+        <f>IF(OR(G$25="",$A33="",NOT(ISNUMBER(G14)),NOT(ISNUMBER(F14)),N(F14)=0),"",G14/F14-1)</f>
+      </c>
+      <c r="H33" s="17">
+        <f>IF(OR(H$25="",$A33="",NOT(ISNUMBER(H14)),NOT(ISNUMBER(G14)),N(G14)=0),"",H14/G14-1)</f>
+      </c>
+      <c r="I33" s="17">
+        <f>IF(OR(I$25="",$A33="",NOT(ISNUMBER(I14)),NOT(ISNUMBER(H14)),N(H14)=0),"",I14/H14-1)</f>
+      </c>
+      <c r="J33" s="17">
+        <f>IF(OR(J$25="",$A33="",NOT(ISNUMBER(J14)),NOT(ISNUMBER(I14)),N(I14)=0),"",J14/I14-1)</f>
+      </c>
+      <c r="K33" s="17">
+        <f>IF(OR(K$25="",$A33="",NOT(ISNUMBER(K14)),NOT(ISNUMBER(J14)),N(J14)=0),"",K14/J14-1)</f>
+      </c>
+      <c r="L33" s="17">
+        <f>IF(OR(L$25="",$A33="",NOT(ISNUMBER(L14)),NOT(ISNUMBER(K14)),N(K14)=0),"",L14/K14-1)</f>
+      </c>
+      <c r="M33" s="17">
+        <f>IF(OR(M$25="",$A33="",NOT(ISNUMBER(M14)),NOT(ISNUMBER(L14)),N(L14)=0),"",M14/L14-1)</f>
+      </c>
+      <c r="N33" s="17">
+        <f>IF(OR(N$25="",$A33="",NOT(ISNUMBER(N14)),NOT(ISNUMBER(M14)),N(M14)=0),"",N14/M14-1)</f>
+      </c>
+      <c r="O33" s="17">
+        <f>IF(OR(O$25="",$A33="",NOT(ISNUMBER(O14)),NOT(ISNUMBER(N14)),N(N14)=0),"",O14/N14-1)</f>
+      </c>
+      <c r="P33" s="17">
+        <f>IF(OR(P$25="",$A33="",NOT(ISNUMBER(P14)),NOT(ISNUMBER(O14)),N(O14)=0),"",P14/O14-1)</f>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <f>IF(OR(A15="",A16=""),"",A15)</f>
+      </c>
+      <c r="B34" s="17">
+        <f>IF(OR(B$25="",$A34="",NOT(ISNUMBER(B15)),NOT(ISNUMBER(A15)),N(A15)=0),"",B15/A15-1)</f>
+      </c>
+      <c r="C34" s="17">
+        <f>IF(OR(C$25="",$A34="",NOT(ISNUMBER(C15)),NOT(ISNUMBER(B15)),N(B15)=0),"",C15/B15-1)</f>
+      </c>
+      <c r="D34" s="17">
+        <f>IF(OR(D$25="",$A34="",NOT(ISNUMBER(D15)),NOT(ISNUMBER(C15)),N(C15)=0),"",D15/C15-1)</f>
+      </c>
+      <c r="E34" s="17">
+        <f>IF(OR(E$25="",$A34="",NOT(ISNUMBER(E15)),NOT(ISNUMBER(D15)),N(D15)=0),"",E15/D15-1)</f>
+      </c>
+      <c r="F34" s="17">
+        <f>IF(OR(F$25="",$A34="",NOT(ISNUMBER(F15)),NOT(ISNUMBER(E15)),N(E15)=0),"",F15/E15-1)</f>
+      </c>
+      <c r="G34" s="17">
+        <f>IF(OR(G$25="",$A34="",NOT(ISNUMBER(G15)),NOT(ISNUMBER(F15)),N(F15)=0),"",G15/F15-1)</f>
+      </c>
+      <c r="H34" s="17">
+        <f>IF(OR(H$25="",$A34="",NOT(ISNUMBER(H15)),NOT(ISNUMBER(G15)),N(G15)=0),"",H15/G15-1)</f>
+      </c>
+      <c r="I34" s="17">
+        <f>IF(OR(I$25="",$A34="",NOT(ISNUMBER(I15)),NOT(ISNUMBER(H15)),N(H15)=0),"",I15/H15-1)</f>
+      </c>
+      <c r="J34" s="17">
+        <f>IF(OR(J$25="",$A34="",NOT(ISNUMBER(J15)),NOT(ISNUMBER(I15)),N(I15)=0),"",J15/I15-1)</f>
+      </c>
+      <c r="K34" s="17">
+        <f>IF(OR(K$25="",$A34="",NOT(ISNUMBER(K15)),NOT(ISNUMBER(J15)),N(J15)=0),"",K15/J15-1)</f>
+      </c>
+      <c r="L34" s="17">
+        <f>IF(OR(L$25="",$A34="",NOT(ISNUMBER(L15)),NOT(ISNUMBER(K15)),N(K15)=0),"",L15/K15-1)</f>
+      </c>
+      <c r="M34" s="17">
+        <f>IF(OR(M$25="",$A34="",NOT(ISNUMBER(M15)),NOT(ISNUMBER(L15)),N(L15)=0),"",M15/L15-1)</f>
+      </c>
+      <c r="N34" s="17">
+        <f>IF(OR(N$25="",$A34="",NOT(ISNUMBER(N15)),NOT(ISNUMBER(M15)),N(M15)=0),"",N15/M15-1)</f>
+      </c>
+      <c r="O34" s="17">
+        <f>IF(OR(O$25="",$A34="",NOT(ISNUMBER(O15)),NOT(ISNUMBER(N15)),N(N15)=0),"",O15/N15-1)</f>
+      </c>
+      <c r="P34" s="17">
+        <f>IF(OR(P$25="",$A34="",NOT(ISNUMBER(P15)),NOT(ISNUMBER(O15)),N(O15)=0),"",P15/O15-1)</f>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <f>IF(OR(A16="",A17=""),"",A16)</f>
+      </c>
+      <c r="B35" s="17">
+        <f>IF(OR(B$25="",$A35="",NOT(ISNUMBER(B16)),NOT(ISNUMBER(A16)),N(A16)=0),"",B16/A16-1)</f>
+      </c>
+      <c r="C35" s="17">
+        <f>IF(OR(C$25="",$A35="",NOT(ISNUMBER(C16)),NOT(ISNUMBER(B16)),N(B16)=0),"",C16/B16-1)</f>
+      </c>
+      <c r="D35" s="17">
+        <f>IF(OR(D$25="",$A35="",NOT(ISNUMBER(D16)),NOT(ISNUMBER(C16)),N(C16)=0),"",D16/C16-1)</f>
+      </c>
+      <c r="E35" s="17">
+        <f>IF(OR(E$25="",$A35="",NOT(ISNUMBER(E16)),NOT(ISNUMBER(D16)),N(D16)=0),"",E16/D16-1)</f>
+      </c>
+      <c r="F35" s="17">
+        <f>IF(OR(F$25="",$A35="",NOT(ISNUMBER(F16)),NOT(ISNUMBER(E16)),N(E16)=0),"",F16/E16-1)</f>
+      </c>
+      <c r="G35" s="17">
+        <f>IF(OR(G$25="",$A35="",NOT(ISNUMBER(G16)),NOT(ISNUMBER(F16)),N(F16)=0),"",G16/F16-1)</f>
+      </c>
+      <c r="H35" s="17">
+        <f>IF(OR(H$25="",$A35="",NOT(ISNUMBER(H16)),NOT(ISNUMBER(G16)),N(G16)=0),"",H16/G16-1)</f>
+      </c>
+      <c r="I35" s="17">
+        <f>IF(OR(I$25="",$A35="",NOT(ISNUMBER(I16)),NOT(ISNUMBER(H16)),N(H16)=0),"",I16/H16-1)</f>
+      </c>
+      <c r="J35" s="17">
+        <f>IF(OR(J$25="",$A35="",NOT(ISNUMBER(J16)),NOT(ISNUMBER(I16)),N(I16)=0),"",J16/I16-1)</f>
+      </c>
+      <c r="K35" s="17">
+        <f>IF(OR(K$25="",$A35="",NOT(ISNUMBER(K16)),NOT(ISNUMBER(J16)),N(J16)=0),"",K16/J16-1)</f>
+      </c>
+      <c r="L35" s="17">
+        <f>IF(OR(L$25="",$A35="",NOT(ISNUMBER(L16)),NOT(ISNUMBER(K16)),N(K16)=0),"",L16/K16-1)</f>
+      </c>
+      <c r="M35" s="17">
+        <f>IF(OR(M$25="",$A35="",NOT(ISNUMBER(M16)),NOT(ISNUMBER(L16)),N(L16)=0),"",M16/L16-1)</f>
+      </c>
+      <c r="N35" s="17">
+        <f>IF(OR(N$25="",$A35="",NOT(ISNUMBER(N16)),NOT(ISNUMBER(M16)),N(M16)=0),"",N16/M16-1)</f>
+      </c>
+      <c r="O35" s="17">
+        <f>IF(OR(O$25="",$A35="",NOT(ISNUMBER(O16)),NOT(ISNUMBER(N16)),N(N16)=0),"",O16/N16-1)</f>
+      </c>
+      <c r="P35" s="17">
+        <f>IF(OR(P$25="",$A35="",NOT(ISNUMBER(P16)),NOT(ISNUMBER(O16)),N(O16)=0),"",P16/O16-1)</f>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <f>IF(OR(A17="",A18=""),"",A17)</f>
+      </c>
+      <c r="B36" s="17">
+        <f>IF(OR(B$25="",$A36="",NOT(ISNUMBER(B17)),NOT(ISNUMBER(A17)),N(A17)=0),"",B17/A17-1)</f>
+      </c>
+      <c r="C36" s="17">
+        <f>IF(OR(C$25="",$A36="",NOT(ISNUMBER(C17)),NOT(ISNUMBER(B17)),N(B17)=0),"",C17/B17-1)</f>
+      </c>
+      <c r="D36" s="17">
+        <f>IF(OR(D$25="",$A36="",NOT(ISNUMBER(D17)),NOT(ISNUMBER(C17)),N(C17)=0),"",D17/C17-1)</f>
+      </c>
+      <c r="E36" s="17">
+        <f>IF(OR(E$25="",$A36="",NOT(ISNUMBER(E17)),NOT(ISNUMBER(D17)),N(D17)=0),"",E17/D17-1)</f>
+      </c>
+      <c r="F36" s="17">
+        <f>IF(OR(F$25="",$A36="",NOT(ISNUMBER(F17)),NOT(ISNUMBER(E17)),N(E17)=0),"",F17/E17-1)</f>
+      </c>
+      <c r="G36" s="17">
+        <f>IF(OR(G$25="",$A36="",NOT(ISNUMBER(G17)),NOT(ISNUMBER(F17)),N(F17)=0),"",G17/F17-1)</f>
+      </c>
+      <c r="H36" s="17">
+        <f>IF(OR(H$25="",$A36="",NOT(ISNUMBER(H17)),NOT(ISNUMBER(G17)),N(G17)=0),"",H17/G17-1)</f>
+      </c>
+      <c r="I36" s="17">
+        <f>IF(OR(I$25="",$A36="",NOT(ISNUMBER(I17)),NOT(ISNUMBER(H17)),N(H17)=0),"",I17/H17-1)</f>
+      </c>
+      <c r="J36" s="17">
+        <f>IF(OR(J$25="",$A36="",NOT(ISNUMBER(J17)),NOT(ISNUMBER(I17)),N(I17)=0),"",J17/I17-1)</f>
+      </c>
+      <c r="K36" s="17">
+        <f>IF(OR(K$25="",$A36="",NOT(ISNUMBER(K17)),NOT(ISNUMBER(J17)),N(J17)=0),"",K17/J17-1)</f>
+      </c>
+      <c r="L36" s="17">
+        <f>IF(OR(L$25="",$A36="",NOT(ISNUMBER(L17)),NOT(ISNUMBER(K17)),N(K17)=0),"",L17/K17-1)</f>
+      </c>
+      <c r="M36" s="17">
+        <f>IF(OR(M$25="",$A36="",NOT(ISNUMBER(M17)),NOT(ISNUMBER(L17)),N(L17)=0),"",M17/L17-1)</f>
+      </c>
+      <c r="N36" s="17">
+        <f>IF(OR(N$25="",$A36="",NOT(ISNUMBER(N17)),NOT(ISNUMBER(M17)),N(M17)=0),"",N17/M17-1)</f>
+      </c>
+      <c r="O36" s="17">
+        <f>IF(OR(O$25="",$A36="",NOT(ISNUMBER(O17)),NOT(ISNUMBER(N17)),N(N17)=0),"",O17/N17-1)</f>
+      </c>
+      <c r="P36" s="17">
+        <f>IF(OR(P$25="",$A36="",NOT(ISNUMBER(P17)),NOT(ISNUMBER(O17)),N(O17)=0),"",P17/O17-1)</f>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <f>IF(OR(A18="",A19=""),"",A18)</f>
+      </c>
+      <c r="B37" s="17">
+        <f>IF(OR(B$25="",$A37="",NOT(ISNUMBER(B18)),NOT(ISNUMBER(A18)),N(A18)=0),"",B18/A18-1)</f>
+      </c>
+      <c r="C37" s="17">
+        <f>IF(OR(C$25="",$A37="",NOT(ISNUMBER(C18)),NOT(ISNUMBER(B18)),N(B18)=0),"",C18/B18-1)</f>
+      </c>
+      <c r="D37" s="17">
+        <f>IF(OR(D$25="",$A37="",NOT(ISNUMBER(D18)),NOT(ISNUMBER(C18)),N(C18)=0),"",D18/C18-1)</f>
+      </c>
+      <c r="E37" s="17">
+        <f>IF(OR(E$25="",$A37="",NOT(ISNUMBER(E18)),NOT(ISNUMBER(D18)),N(D18)=0),"",E18/D18-1)</f>
+      </c>
+      <c r="F37" s="17">
+        <f>IF(OR(F$25="",$A37="",NOT(ISNUMBER(F18)),NOT(ISNUMBER(E18)),N(E18)=0),"",F18/E18-1)</f>
+      </c>
+      <c r="G37" s="17">
+        <f>IF(OR(G$25="",$A37="",NOT(ISNUMBER(G18)),NOT(ISNUMBER(F18)),N(F18)=0),"",G18/F18-1)</f>
+      </c>
+      <c r="H37" s="17">
+        <f>IF(OR(H$25="",$A37="",NOT(ISNUMBER(H18)),NOT(ISNUMBER(G18)),N(G18)=0),"",H18/G18-1)</f>
+      </c>
+      <c r="I37" s="17">
+        <f>IF(OR(I$25="",$A37="",NOT(ISNUMBER(I18)),NOT(ISNUMBER(H18)),N(H18)=0),"",I18/H18-1)</f>
+      </c>
+      <c r="J37" s="17">
+        <f>IF(OR(J$25="",$A37="",NOT(ISNUMBER(J18)),NOT(ISNUMBER(I18)),N(I18)=0),"",J18/I18-1)</f>
+      </c>
+      <c r="K37" s="17">
+        <f>IF(OR(K$25="",$A37="",NOT(ISNUMBER(K18)),NOT(ISNUMBER(J18)),N(J18)=0),"",K18/J18-1)</f>
+      </c>
+      <c r="L37" s="17">
+        <f>IF(OR(L$25="",$A37="",NOT(ISNUMBER(L18)),NOT(ISNUMBER(K18)),N(K18)=0),"",L18/K18-1)</f>
+      </c>
+      <c r="M37" s="17">
+        <f>IF(OR(M$25="",$A37="",NOT(ISNUMBER(M18)),NOT(ISNUMBER(L18)),N(L18)=0),"",M18/L18-1)</f>
+      </c>
+      <c r="N37" s="17">
+        <f>IF(OR(N$25="",$A37="",NOT(ISNUMBER(N18)),NOT(ISNUMBER(M18)),N(M18)=0),"",N18/M18-1)</f>
+      </c>
+      <c r="O37" s="17">
+        <f>IF(OR(O$25="",$A37="",NOT(ISNUMBER(O18)),NOT(ISNUMBER(N18)),N(N18)=0),"",O18/N18-1)</f>
+      </c>
+      <c r="P37" s="17">
+        <f>IF(OR(P$25="",$A37="",NOT(ISNUMBER(P18)),NOT(ISNUMBER(O18)),N(O18)=0),"",P18/O18-1)</f>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <f>IF(OR(A19="",A20=""),"",A19)</f>
+      </c>
+      <c r="B38" s="17">
+        <f>IF(OR(B$25="",$A38="",NOT(ISNUMBER(B19)),NOT(ISNUMBER(A19)),N(A19)=0),"",B19/A19-1)</f>
+      </c>
+      <c r="C38" s="17">
+        <f>IF(OR(C$25="",$A38="",NOT(ISNUMBER(C19)),NOT(ISNUMBER(B19)),N(B19)=0),"",C19/B19-1)</f>
+      </c>
+      <c r="D38" s="17">
+        <f>IF(OR(D$25="",$A38="",NOT(ISNUMBER(D19)),NOT(ISNUMBER(C19)),N(C19)=0),"",D19/C19-1)</f>
+      </c>
+      <c r="E38" s="17">
+        <f>IF(OR(E$25="",$A38="",NOT(ISNUMBER(E19)),NOT(ISNUMBER(D19)),N(D19)=0),"",E19/D19-1)</f>
+      </c>
+      <c r="F38" s="17">
+        <f>IF(OR(F$25="",$A38="",NOT(ISNUMBER(F19)),NOT(ISNUMBER(E19)),N(E19)=0),"",F19/E19-1)</f>
+      </c>
+      <c r="G38" s="17">
+        <f>IF(OR(G$25="",$A38="",NOT(ISNUMBER(G19)),NOT(ISNUMBER(F19)),N(F19)=0),"",G19/F19-1)</f>
+      </c>
+      <c r="H38" s="17">
+        <f>IF(OR(H$25="",$A38="",NOT(ISNUMBER(H19)),NOT(ISNUMBER(G19)),N(G19)=0),"",H19/G19-1)</f>
+      </c>
+      <c r="I38" s="17">
+        <f>IF(OR(I$25="",$A38="",NOT(ISNUMBER(I19)),NOT(ISNUMBER(H19)),N(H19)=0),"",I19/H19-1)</f>
+      </c>
+      <c r="J38" s="17">
+        <f>IF(OR(J$25="",$A38="",NOT(ISNUMBER(J19)),NOT(ISNUMBER(I19)),N(I19)=0),"",J19/I19-1)</f>
+      </c>
+      <c r="K38" s="17">
+        <f>IF(OR(K$25="",$A38="",NOT(ISNUMBER(K19)),NOT(ISNUMBER(J19)),N(J19)=0),"",K19/J19-1)</f>
+      </c>
+      <c r="L38" s="17">
+        <f>IF(OR(L$25="",$A38="",NOT(ISNUMBER(L19)),NOT(ISNUMBER(K19)),N(K19)=0),"",L19/K19-1)</f>
+      </c>
+      <c r="M38" s="17">
+        <f>IF(OR(M$25="",$A38="",NOT(ISNUMBER(M19)),NOT(ISNUMBER(L19)),N(L19)=0),"",M19/L19-1)</f>
+      </c>
+      <c r="N38" s="17">
+        <f>IF(OR(N$25="",$A38="",NOT(ISNUMBER(N19)),NOT(ISNUMBER(M19)),N(M19)=0),"",N19/M19-1)</f>
+      </c>
+      <c r="O38" s="17">
+        <f>IF(OR(O$25="",$A38="",NOT(ISNUMBER(O19)),NOT(ISNUMBER(N19)),N(N19)=0),"",O19/N19-1)</f>
+      </c>
+      <c r="P38" s="17">
+        <f>IF(OR(P$25="",$A38="",NOT(ISNUMBER(P19)),NOT(ISNUMBER(O19)),N(O19)=0),"",P19/O19-1)</f>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <f>IF(OR(A20="",A21=""),"",A20)</f>
+      </c>
+      <c r="B39" s="17">
+        <f>IF(OR(B$25="",$A39="",NOT(ISNUMBER(B20)),NOT(ISNUMBER(A20)),N(A20)=0),"",B20/A20-1)</f>
+      </c>
+      <c r="C39" s="17">
+        <f>IF(OR(C$25="",$A39="",NOT(ISNUMBER(C20)),NOT(ISNUMBER(B20)),N(B20)=0),"",C20/B20-1)</f>
+      </c>
+      <c r="D39" s="17">
+        <f>IF(OR(D$25="",$A39="",NOT(ISNUMBER(D20)),NOT(ISNUMBER(C20)),N(C20)=0),"",D20/C20-1)</f>
+      </c>
+      <c r="E39" s="17">
+        <f>IF(OR(E$25="",$A39="",NOT(ISNUMBER(E20)),NOT(ISNUMBER(D20)),N(D20)=0),"",E20/D20-1)</f>
+      </c>
+      <c r="F39" s="17">
+        <f>IF(OR(F$25="",$A39="",NOT(ISNUMBER(F20)),NOT(ISNUMBER(E20)),N(E20)=0),"",F20/E20-1)</f>
+      </c>
+      <c r="G39" s="17">
+        <f>IF(OR(G$25="",$A39="",NOT(ISNUMBER(G20)),NOT(ISNUMBER(F20)),N(F20)=0),"",G20/F20-1)</f>
+      </c>
+      <c r="H39" s="17">
+        <f>IF(OR(H$25="",$A39="",NOT(ISNUMBER(H20)),NOT(ISNUMBER(G20)),N(G20)=0),"",H20/G20-1)</f>
+      </c>
+      <c r="I39" s="17">
+        <f>IF(OR(I$25="",$A39="",NOT(ISNUMBER(I20)),NOT(ISNUMBER(H20)),N(H20)=0),"",I20/H20-1)</f>
+      </c>
+      <c r="J39" s="17">
+        <f>IF(OR(J$25="",$A39="",NOT(ISNUMBER(J20)),NOT(ISNUMBER(I20)),N(I20)=0),"",J20/I20-1)</f>
+      </c>
+      <c r="K39" s="17">
+        <f>IF(OR(K$25="",$A39="",NOT(ISNUMBER(K20)),NOT(ISNUMBER(J20)),N(J20)=0),"",K20/J20-1)</f>
+      </c>
+      <c r="L39" s="17">
+        <f>IF(OR(L$25="",$A39="",NOT(ISNUMBER(L20)),NOT(ISNUMBER(K20)),N(K20)=0),"",L20/K20-1)</f>
+      </c>
+      <c r="M39" s="17">
+        <f>IF(OR(M$25="",$A39="",NOT(ISNUMBER(M20)),NOT(ISNUMBER(L20)),N(L20)=0),"",M20/L20-1)</f>
+      </c>
+      <c r="N39" s="17">
+        <f>IF(OR(N$25="",$A39="",NOT(ISNUMBER(N20)),NOT(ISNUMBER(M20)),N(M20)=0),"",N20/M20-1)</f>
+      </c>
+      <c r="O39" s="17">
+        <f>IF(OR(O$25="",$A39="",NOT(ISNUMBER(O20)),NOT(ISNUMBER(N20)),N(N20)=0),"",O20/N20-1)</f>
+      </c>
+      <c r="P39" s="17">
+        <f>IF(OR(P$25="",$A39="",NOT(ISNUMBER(P20)),NOT(ISNUMBER(O20)),N(O20)=0),"",P20/O20-1)</f>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <f>IF(OR(A21="",A22=""),"",A21)</f>
+      </c>
+      <c r="B40" s="17">
+        <f>IF(OR(B$25="",$A40="",NOT(ISNUMBER(B21)),NOT(ISNUMBER(A21)),N(A21)=0),"",B21/A21-1)</f>
+      </c>
+      <c r="C40" s="17">
+        <f>IF(OR(C$25="",$A40="",NOT(ISNUMBER(C21)),NOT(ISNUMBER(B21)),N(B21)=0),"",C21/B21-1)</f>
+      </c>
+      <c r="D40" s="17">
+        <f>IF(OR(D$25="",$A40="",NOT(ISNUMBER(D21)),NOT(ISNUMBER(C21)),N(C21)=0),"",D21/C21-1)</f>
+      </c>
+      <c r="E40" s="17">
+        <f>IF(OR(E$25="",$A40="",NOT(ISNUMBER(E21)),NOT(ISNUMBER(D21)),N(D21)=0),"",E21/D21-1)</f>
+      </c>
+      <c r="F40" s="17">
+        <f>IF(OR(F$25="",$A40="",NOT(ISNUMBER(F21)),NOT(ISNUMBER(E21)),N(E21)=0),"",F21/E21-1)</f>
+      </c>
+      <c r="G40" s="17">
+        <f>IF(OR(G$25="",$A40="",NOT(ISNUMBER(G21)),NOT(ISNUMBER(F21)),N(F21)=0),"",G21/F21-1)</f>
+      </c>
+      <c r="H40" s="17">
+        <f>IF(OR(H$25="",$A40="",NOT(ISNUMBER(H21)),NOT(ISNUMBER(G21)),N(G21)=0),"",H21/G21-1)</f>
+      </c>
+      <c r="I40" s="17">
+        <f>IF(OR(I$25="",$A40="",NOT(ISNUMBER(I21)),NOT(ISNUMBER(H21)),N(H21)=0),"",I21/H21-1)</f>
+      </c>
+      <c r="J40" s="17">
+        <f>IF(OR(J$25="",$A40="",NOT(ISNUMBER(J21)),NOT(ISNUMBER(I21)),N(I21)=0),"",J21/I21-1)</f>
+      </c>
+      <c r="K40" s="17">
+        <f>IF(OR(K$25="",$A40="",NOT(ISNUMBER(K21)),NOT(ISNUMBER(J21)),N(J21)=0),"",K21/J21-1)</f>
+      </c>
+      <c r="L40" s="17">
+        <f>IF(OR(L$25="",$A40="",NOT(ISNUMBER(L21)),NOT(ISNUMBER(K21)),N(K21)=0),"",L21/K21-1)</f>
+      </c>
+      <c r="M40" s="17">
+        <f>IF(OR(M$25="",$A40="",NOT(ISNUMBER(M21)),NOT(ISNUMBER(L21)),N(L21)=0),"",M21/L21-1)</f>
+      </c>
+      <c r="N40" s="17">
+        <f>IF(OR(N$25="",$A40="",NOT(ISNUMBER(N21)),NOT(ISNUMBER(M21)),N(M21)=0),"",N21/M21-1)</f>
+      </c>
+      <c r="O40" s="17">
+        <f>IF(OR(O$25="",$A40="",NOT(ISNUMBER(O21)),NOT(ISNUMBER(N21)),N(N21)=0),"",O21/N21-1)</f>
+      </c>
+      <c r="P40" s="17">
+        <f>IF(OR(P$25="",$A40="",NOT(ISNUMBER(P21)),NOT(ISNUMBER(O21)),N(O21)=0),"",P21/O21-1)</f>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total (meses comparables)</t>
+        </is>
+      </c>
+      <c r="B41" s="17">
+        <f>IF(B$25="","",IFERROR(SUMPRODUCT(ISNUMBER(B7:B21)*ISNUMBER(A7:A21)*($A8:$A22&lt;&gt;""),B7:B21)/SUMPRODUCT(ISNUMBER(B7:B21)*ISNUMBER(A7:A21)*($A8:$A22&lt;&gt;""),A7:A21)-1,""))</f>
+      </c>
+      <c r="C41" s="17">
+        <f>IF(C$25="","",IFERROR(SUMPRODUCT(ISNUMBER(C7:C21)*ISNUMBER(B7:B21)*($A8:$A22&lt;&gt;""),C7:C21)/SUMPRODUCT(ISNUMBER(C7:C21)*ISNUMBER(B7:B21)*($A8:$A22&lt;&gt;""),B7:B21)-1,""))</f>
+      </c>
+      <c r="D41" s="17">
+        <f>IF(D$25="","",IFERROR(SUMPRODUCT(ISNUMBER(D7:D21)*ISNUMBER(C7:C21)*($A8:$A22&lt;&gt;""),D7:D21)/SUMPRODUCT(ISNUMBER(D7:D21)*ISNUMBER(C7:C21)*($A8:$A22&lt;&gt;""),C7:C21)-1,""))</f>
+      </c>
+      <c r="E41" s="17">
+        <f>IF(E$25="","",IFERROR(SUMPRODUCT(ISNUMBER(E7:E21)*ISNUMBER(D7:D21)*($A8:$A22&lt;&gt;""),E7:E21)/SUMPRODUCT(ISNUMBER(E7:E21)*ISNUMBER(D7:D21)*($A8:$A22&lt;&gt;""),D7:D21)-1,""))</f>
+      </c>
+      <c r="F41" s="17">
+        <f>IF(F$25="","",IFERROR(SUMPRODUCT(ISNUMBER(F7:F21)*ISNUMBER(E7:E21)*($A8:$A22&lt;&gt;""),F7:F21)/SUMPRODUCT(ISNUMBER(F7:F21)*ISNUMBER(E7:E21)*($A8:$A22&lt;&gt;""),E7:E21)-1,""))</f>
+      </c>
+      <c r="G41" s="17">
+        <f>IF(G$25="","",IFERROR(SUMPRODUCT(ISNUMBER(G7:G21)*ISNUMBER(F7:F21)*($A8:$A22&lt;&gt;""),G7:G21)/SUMPRODUCT(ISNUMBER(G7:G21)*ISNUMBER(F7:F21)*($A8:$A22&lt;&gt;""),F7:F21)-1,""))</f>
+      </c>
+      <c r="H41" s="17">
+        <f>IF(H$25="","",IFERROR(SUMPRODUCT(ISNUMBER(H7:H21)*ISNUMBER(G7:G21)*($A8:$A22&lt;&gt;""),H7:H21)/SUMPRODUCT(ISNUMBER(H7:H21)*ISNUMBER(G7:G21)*($A8:$A22&lt;&gt;""),G7:G21)-1,""))</f>
+      </c>
+      <c r="I41" s="17">
+        <f>IF(I$25="","",IFERROR(SUMPRODUCT(ISNUMBER(I7:I21)*ISNUMBER(H7:H21)*($A8:$A22&lt;&gt;""),I7:I21)/SUMPRODUCT(ISNUMBER(I7:I21)*ISNUMBER(H7:H21)*($A8:$A22&lt;&gt;""),H7:H21)-1,""))</f>
+      </c>
+      <c r="J41" s="17">
+        <f>IF(J$25="","",IFERROR(SUMPRODUCT(ISNUMBER(J7:J21)*ISNUMBER(I7:I21)*($A8:$A22&lt;&gt;""),J7:J21)/SUMPRODUCT(ISNUMBER(J7:J21)*ISNUMBER(I7:I21)*($A8:$A22&lt;&gt;""),I7:I21)-1,""))</f>
+      </c>
+      <c r="K41" s="17">
+        <f>IF(K$25="","",IFERROR(SUMPRODUCT(ISNUMBER(K7:K21)*ISNUMBER(J7:J21)*($A8:$A22&lt;&gt;""),K7:K21)/SUMPRODUCT(ISNUMBER(K7:K21)*ISNUMBER(J7:J21)*($A8:$A22&lt;&gt;""),J7:J21)-1,""))</f>
+      </c>
+      <c r="L41" s="17">
+        <f>IF(L$25="","",IFERROR(SUMPRODUCT(ISNUMBER(L7:L21)*ISNUMBER(K7:K21)*($A8:$A22&lt;&gt;""),L7:L21)/SUMPRODUCT(ISNUMBER(L7:L21)*ISNUMBER(K7:K21)*($A8:$A22&lt;&gt;""),K7:K21)-1,""))</f>
+      </c>
+      <c r="M41" s="17">
+        <f>IF(M$25="","",IFERROR(SUMPRODUCT(ISNUMBER(M7:M21)*ISNUMBER(L7:L21)*($A8:$A22&lt;&gt;""),M7:M21)/SUMPRODUCT(ISNUMBER(M7:M21)*ISNUMBER(L7:L21)*($A8:$A22&lt;&gt;""),L7:L21)-1,""))</f>
+      </c>
+      <c r="N41" s="17">
+        <f>IF(N$25="","",IFERROR(SUMPRODUCT(ISNUMBER(N7:N21)*ISNUMBER(M7:M21)*($A8:$A22&lt;&gt;""),N7:N21)/SUMPRODUCT(ISNUMBER(N7:N21)*ISNUMBER(M7:M21)*($A8:$A22&lt;&gt;""),M7:M21)-1,""))</f>
+      </c>
+      <c r="O41" s="17">
+        <f>IF(O$25="","",IFERROR(SUMPRODUCT(ISNUMBER(O7:O21)*ISNUMBER(N7:N21)*($A8:$A22&lt;&gt;""),O7:O21)/SUMPRODUCT(ISNUMBER(O7:O21)*ISNUMBER(N7:N21)*($A8:$A22&lt;&gt;""),N7:N21)-1,""))</f>
+      </c>
+      <c r="P41" s="17">
+        <f>IF(P$25="","",IFERROR(SUMPRODUCT(ISNUMBER(P7:P21)*ISNUMBER(O7:O21)*($A8:$A22&lt;&gt;""),P7:P21)/SUMPRODUCT(ISNUMBER(P7:P21)*ISNUMBER(O7:O21)*($A8:$A22&lt;&gt;""),O7:O21)-1,""))</f>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B26:P41">
+    <cfRule type="cellIs" dxfId="19" priority="1" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D558"/>

</xml_diff>

<commit_message>
Amplía las descripciones de las hojas dinámicas de la plantilla xlsx
Sustituye las descripciones de una línea de Productos, MiInflación,
T_Precio, T_Cantidad, Mes, Año, Último, Evolucion-€ y Evolucion-N por
textos cortos que explican qué muestra cada tabla y cómo usar sus
filtros, ajustados a la configuración real de cada tabla dinámica (p.
ej. Mes suma unidades, no promedia, y su filtro fecha junta el mismo
mes de todos los años; Evolucion-N muestra la evolución año a año).
Incluye las advertencias relevantes: los productos a peso no tienen
precio por unidad y cuentan 1 unidad por compra.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -176,28 +176,28 @@
     <t>Suma de unidades</t>
   </si>
   <si>
-    <t>Listado de productos comprados agrupados por el número de veces comprado. Incluye promedios sobre el producto</t>
+    <t>Productos ordenados por el nº de veces que se han comprado (cada línea de ticket cuenta una vez), con su precio medio por unidad. Los productos a peso no tienen precio por unidad y salen vacíos.</t>
   </si>
   <si>
-    <t>Número de productos comprados al mes. Con gráfica</t>
+    <t>Unidades compradas por año y mes, en tabla y gráfica. El filtro id permite ver uno o varios productos; sin filtro suma todos. Los productos a peso cuentan 1 unidad por compra.</t>
   </si>
   <si>
-    <t>Dinero gastado al mes. Con gráfica</t>
+    <t>Gasto total (€) por año y mes, en tabla y gráfica, sumando todas las compras. Sirve para ver qué meses se gasta más y cómo evoluciona el gasto.</t>
   </si>
   <si>
-    <t>Ultima vez que se compró un producto</t>
+    <t>Fecha de la última compra de cada producto. Sirve para detectar productos que llevan más tiempo del habitual sin comprarse.</t>
   </si>
   <si>
-    <t>Evolución del precio de un producto promediado al mes. En el selector se fija el producto y permite ver como ha evolucionado su precio con el tiempo</t>
+    <t>Precio medio por unidad de un producto, mes a mes, en tabla y gráfica. Elige un único producto en el filtro id (con varios la media los mezcla). Los productos a peso no tienen precio por unidad.</t>
   </si>
   <si>
-    <t>Promedio por mes de unidades de un producto. Con selectores para fijar el producto y el mes</t>
+    <t>Unidades compradas de cada producto, de más a menos. El filtro fecha elige un mes del año (suma ese mes de todos los años) para ver qué se compra más en cada época.</t>
   </si>
   <si>
-    <t>Número de productos comprados al año. Especie de bolsa de la compara anual. Muestra cuanto se ha gastado en ese producto al año</t>
+    <t>La cesta de la compra de cada año: qué productos se compraron, cuántas veces (líneas de ticket) y cuánto se gastó (€) en cada uno.</t>
   </si>
   <si>
-    <t>Esto se un cáculo de la inflación sufrida por los productos comprados. No es la inflación calculada por el INE</t>
+    <t>Inflación de tu propia cesta de la compra (no es el IPC del INE): % de variación de precios frente al año base. Laspeyres pondera con lo comprado el año base; Paasche, con lo comprado cada año. Solo cuentan los productos comprados en ambos años (Productos coincidentes).</t>
   </si>
   <si>
     <t>Año</t>
@@ -218,7 +218,7 @@
     <t>Productos coincidentes</t>
   </si>
   <si>
-    <t>Evolución de la cantidad de productos comprados en un año. En el selector se fija el producto y permite ver como ha evolucionadoel número de productos comprados</t>
+    <t>Unidades compradas de un producto cada año, en tabla y gráfica. Elige el producto en el filtro id (sin filtro suma todos). El primer y el último año pueden estar incompletos.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Quita la preselección de productos en la hoja Pareto de la plantilla xlsx
El elemento "(en blanco)" del campo id estaba marcado como oculto, y
Excel lo trataba como un filtro manual: al refrescar la caché con los
datos reales solo dejaba visibles los dos productos de ejemplo de la
plantilla y ocultaba el resto. Ahora el campo no tiene ningún elemento
oculto y salen todos los productos; la fila "(en blanco)" aparece al
final sin afectar al % acumulado ni a las clases A/B/C.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -5241,13 +5241,13 @@
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámicaPareto" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A7:D10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <location ref="A7:D11" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
         <item x="1"/>
-        <item x="2" h="1"/>
+        <item x="2"/>
       </items>
       <autoSortScope>
         <pivotArea dataOnly="0" outline="0" fieldPosition="0">
@@ -5294,12 +5294,15 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="4">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
     </i>
     <i t="grand">
       <x/>

</xml_diff>

<commit_message>
Añade hora de compra y número de factura a la tabla de datos
La columna fecha de Datos (y del CSV) pasa a incluir hora y minuto, y se
añade la columna factura con el número de factura simplificada del
ticket, que permite distinguir dos compras del mismo día. En el xlsx la
fecha se escribe como fecha de Excel con la hora como fracción del día y
con un nuevo estilo "dd/mm/yyyy hh:mm" (cellXfs 18) en la plantilla.

La caché de las tablas dinámicas gana el campo factura (antes del campo
agrupado Años, renumerado en todas las tablas) y pasa a leer el nombre
definido DatosTablaDinamica, un OFFSET que abarca tantas columnas como
cabeceras haya en la fila 1: así una columna nueva entra en las tablas
dinámicas sin ampliar el rango. No se usa un rango fijo con columnas de
sobra porque Excel rechaza campos sin cabecera al refrescar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -26,9 +26,10 @@
     <sheet name="Evolucion-N" sheetId="17" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Datos!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Datos!$A$1:$H$3</definedName>
     <definedName name="compras_mercadona" localSheetId="0">Datos!#REF!</definedName>
     <definedName name="export_personal_dataa" localSheetId="0">Datos!$A$1:$G$3</definedName>
+    <definedName name="DatosTablaDinamica">OFFSET(Datos!$A$1,0,0,1048576,COUNTA(Datos!$1:$1))</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
   <pivotCaches>
@@ -225,8 +226,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -318,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -343,6 +345,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4310,9 +4313,9 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="dserrada@gmail.com" refreshedDate="46277.655617592594" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="3">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:G1048576" sheet="Datos"/>
+    <worksheetSource name="DatosTablaDinamica"/>
   </cacheSource>
-  <cacheFields count="8">
+  <cacheFields count="9">
     <cacheField name="id" numFmtId="0">
       <sharedItems containsBlank="1" count="3">
         <s v="COCKTAIL RODEO"/>
@@ -4326,7 +4329,7 @@
         <d v="2023-06-17T00:00:00"/>
         <m/>
       </sharedItems>
-      <fieldGroup par="7" base="1">
+      <fieldGroup par="8" base="1">
         <rangePr groupBy="months" startDate="2023-06-16T00:00:00" endDate="2023-06-18T00:00:00"/>
         <groupItems count="14">
           <s v="(en blanco)"/>
@@ -4361,6 +4364,13 @@
     <cacheField name="precio" numFmtId="0">
       <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0.48" maxValue="3.5"/>
     </cacheField>
+    <cacheField name="factura" numFmtId="0">
+      <sharedItems containsBlank="1" count="3">
+        <s v="0000-000-000001"/>
+        <s v="0000-000-000002"/>
+        <m/>
+      </sharedItems>
+    </cacheField>
     <cacheField name="Años" numFmtId="0" databaseField="0">
       <fieldGroup base="1">
         <rangePr groupBy="years" startDate="2023-06-16T00:00:00" endDate="2023-06-18T00:00:00"/>
@@ -4390,6 +4400,7 @@
     <m/>
     <m/>
     <n v="3.5"/>
+    <x v="0"/>
   </r>
   <r>
     <x v="1"/>
@@ -4399,6 +4410,7 @@
     <m/>
     <m/>
     <n v="0.48"/>
+    <x v="1"/>
   </r>
   <r>
     <x v="2"/>
@@ -4408,6 +4420,7 @@
     <m/>
     <m/>
     <m/>
+    <x v="2"/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -4415,7 +4428,7 @@
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending" defaultSubtotal="0">
       <items count="3">
         <item x="1"/>
@@ -4453,6 +4466,7 @@
     </pivotField>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
@@ -4508,7 +4522,7 @@
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámicaInteranual" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="14">
@@ -4533,6 +4547,7 @@
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisCol" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -4553,7 +4568,7 @@
     </i>
   </rowItems>
   <colFields count="1">
-    <field x="7"/>
+    <field x="8"/>
   </colFields>
   <colItems count="2">
     <i>
@@ -4578,7 +4593,7 @@
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="15">
@@ -4604,6 +4619,7 @@
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -4613,7 +4629,7 @@
     </pivotField>
   </pivotFields>
   <rowFields count="2">
-    <field x="7"/>
+    <field x="8"/>
     <field x="1"/>
   </rowFields>
   <rowItems count="5">
@@ -4682,7 +4698,7 @@
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="1"/>
@@ -4714,6 +4730,7 @@
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -4723,7 +4740,7 @@
     </pivotField>
   </pivotFields>
   <rowFields count="2">
-    <field x="7"/>
+    <field x="8"/>
     <field x="1"/>
   </rowFields>
   <rowItems count="5">
@@ -4795,7 +4812,7 @@
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A7:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0" sortType="descending" defaultSubtotal="0">
       <items count="3">
         <item x="1"/>
@@ -4832,6 +4849,7 @@
       </items>
     </pivotField>
     <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
@@ -4893,7 +4911,7 @@
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:C10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending">
       <items count="4">
         <item x="1"/>
@@ -4935,6 +4953,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -4944,7 +4963,7 @@
     </pivotField>
   </pivotFields>
   <rowFields count="2">
-    <field x="7"/>
+    <field x="8"/>
     <field x="0"/>
   </rowFields>
   <rowItems count="6">
@@ -4994,7 +5013,7 @@
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisRow" multipleItemSelectionAllowed="1" showAll="0" sortType="descending">
       <items count="4">
         <item x="1"/>
@@ -5036,6 +5055,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -5079,7 +5099,7 @@
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A6:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item x="1"/>
@@ -5112,6 +5132,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -5121,7 +5142,7 @@
     </pivotField>
   </pivotFields>
   <rowFields count="2">
-    <field x="7"/>
+    <field x="8"/>
     <field x="1"/>
   </rowFields>
   <rowItems count="5">
@@ -5173,7 +5194,7 @@
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A6:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item x="1"/>
@@ -5188,6 +5209,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -5197,7 +5219,7 @@
     </pivotField>
   </pivotFields>
   <rowFields count="1">
-    <field x="7"/>
+    <field x="8"/>
   </rowFields>
   <rowItems count="3">
     <i>
@@ -5242,7 +5264,7 @@
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámicaPareto" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A7:D11" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="8">
+  <pivotFields count="9">
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="descending" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -5283,6 +5305,7 @@
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
       <items count="3">
         <item x="0"/>
@@ -5323,7 +5346,7 @@
     </i>
   </colItems>
   <pageFields count="1">
-    <pageField fld="7" hier="-1"/>
+    <pageField fld="8" hier="-1"/>
   </pageFields>
   <dataFields count="3">
     <dataField name="Gasto" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
@@ -5602,19 +5625,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="18" customWidth="1"/>
     <col min="3" max="3" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -5636,12 +5660,17 @@
       <c r="G1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>factura</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="18">
         <v>45093</v>
       </c>
       <c r="C2">
@@ -5653,12 +5682,17 @@
       <c r="G2">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0000-000-000001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="18">
         <v>45094</v>
       </c>
       <c r="C3">
@@ -5670,9 +5704,14 @@
       <c r="G3">
         <v>0.48</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0000-000-000002</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:H3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Añade las hojas Facturas y FacturasUnid a la plantilla xlsx
XlsxDatosWriter rellena la nueva hoja Facturas con una fila por ticket
(factura, fecha, año, líneas, unidades, importe). La hoja FacturasUnid
es una tabla dinámica con caché propia que agrupa las facturas por
unidades de 10 en 10, y sustituye a la hoja hecha a mano con Power Query.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -13,6 +13,7 @@
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="6" r:id="rId1"/>
+    <sheet name="Facturas" sheetId="20" r:id="rId17"/>
     <sheet name="Productos" sheetId="7" r:id="rId2"/>
     <sheet name="Pareto" sheetId="18" r:id="rId15"/>
     <sheet name="MiInflación" sheetId="16" r:id="rId3"/>
@@ -24,16 +25,19 @@
     <sheet name="Último" sheetId="13" r:id="rId8"/>
     <sheet name="Evolucion-€" sheetId="14" r:id="rId9"/>
     <sheet name="Evolucion-N" sheetId="17" r:id="rId10"/>
+    <sheet name="FacturasUnid" sheetId="21" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Datos!$A$1:$H$3</definedName>
     <definedName name="compras_mercadona" localSheetId="0">Datos!#REF!</definedName>
     <definedName name="export_personal_dataa" localSheetId="0">Datos!$A$1:$G$3</definedName>
     <definedName name="DatosTablaDinamica">OFFSET(Datos!$A$1,0,0,1048576,COUNTA(Datos!$1:$1))</definedName>
+    <definedName name="FacturasTablaDinamica">OFFSET(Facturas!$A$1,0,0,COUNTA(Facturas!$A:$A),COUNTA(Facturas!$1:$1))</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
   <pivotCaches>
     <pivotCache cacheId="4" r:id="rId11"/>
+    <pivotCache cacheId="5" r:id="rId19"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -4390,6 +4394,44 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="2">
+  <cacheSource type="worksheet">
+    <worksheetSource name="FacturasTablaDinamica"/>
+  </cacheSource>
+  <cacheFields count="6">
+    <cacheField name="factura" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="fecha" numFmtId="165">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2023-06-16T00:00:00" maxDate="2023-06-17T00:00:00"/>
+    </cacheField>
+    <cacheField name="año" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2023" maxValue="2023" count="1">
+        <n v="2023"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="lineas" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="1"/>
+    </cacheField>
+    <cacheField name="unidades" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="2"/>
+      <fieldGroup base="4">
+        <rangePr autoStart="0" startNum="0" endNum="2" groupInterval="10"/>
+        <groupItems count="3">
+          <s v="&lt;0"/>
+          <s v="0-9"/>
+          <s v="&gt;10"/>
+        </groupItems>
+      </fieldGroup>
+    </cacheField>
+    <cacheField name="importe" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.48" maxValue="3.5"/>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="3">
   <r>
@@ -4421,6 +4463,27 @@
     <m/>
     <m/>
     <x v="2"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="2">
+  <r>
+    <s v="0000-000-000001"/>
+    <d v="2023-06-16T00:00:00"/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="2"/>
+    <n v="3.5"/>
+  </r>
+  <r>
+    <s v="0000-000-000002"/>
+    <d v="2023-06-17T00:00:00"/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="1"/>
+    <n v="0.48"/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -4587,6 +4650,66 @@
       <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
     </ext>
   </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámicaFacturasUnid" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Unidades por ticket">
+  <location ref="A7:D9" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="6">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="2" hier="-1"/>
+  </pageFields>
+  <dataFields count="3">
+    <dataField name="Facturas" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="% facturas" fld="0" subtotal="count" showDataAs="percentOfCol" baseField="0" baseItem="0" numFmtId="10"/>
+    <dataField name="Importe medio" fld="5" subtotal="average" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
 </file>
 
@@ -22799,6 +22922,168 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="18" customWidth="1"/>
+    <col min="3" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" style="6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">factura</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fecha</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">año</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lineas</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unidades</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">importe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000-000-000001</t>
+        </is>
+      </c>
+      <c r="B2" s="18">
+        <v>45093</v>
+      </c>
+      <c r="C2">
+        <v>2023</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2" s="6">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000-000-000002</t>
+        </is>
+      </c>
+      <c r="B3" s="18">
+        <v>45094</v>
+      </c>
+      <c r="C3">
+        <v>2023</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0.48</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="4" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facturas por número de unidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuántos tickets hay según las unidades compradas en cada uno (de 10 en 10: 0-9, 10-19...), con su peso sobre el total y el importe medio del ticket en ese rango. Separa las compras pequeñas de reposición de las compras grandes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Un producto a peso cuenta como 1 unidad. Para cambiar el tamaño del rango: botón derecho sobre la columna de rangos &gt; Agrupar. Datos de origen: hoja Facturas (una fila por ticket).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">año</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(Todas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unidades por ticket</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facturas</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% facturas</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Importe medio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D558"/>

</xml_diff>

<commit_message>
Añade la hoja MapaCalor (gasto por producto y mes) a la plantilla xlsx
Tabla dinámica con los 50 productos de más gasto en filas y año-mes en
columnas, con el gasto mensual en euros redondeados y una escala de color
asociada a la propia tabla para que Excel no la pierda al refrescarla.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
+++ b/projects/ticket-digital-data/src/main/resources/Mercadona-base.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Pareto" sheetId="18" r:id="rId15"/>
     <sheet name="MiInflación" sheetId="16" r:id="rId3"/>
     <sheet name="Interanual" sheetId="19" r:id="rId16"/>
+    <sheet name="MapaCalor" sheetId="22" r:id="rId20"/>
     <sheet name="T_Precio" sheetId="8" r:id="rId4"/>
     <sheet name="T_Cantidad" sheetId="15" r:id="rId5"/>
     <sheet name="Mes" sheetId="10" r:id="rId6"/>
@@ -4713,6 +4714,113 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámicaMapaCalor" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A6:B10" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisRow" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0" defaultSubtotal="0">
+      <items count="14">
+        <item x="0" h="1"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisCol" showAll="0" defaultSubtotal="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+  </rowItems>
+  <colFields count="2">
+    <field x="8"/>
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+      <x v="6"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Gasto" fld="6" baseField="0" baseItem="0" numFmtId="1"/>
+  </dataFields>
+  <conditionalFormats count="1">
+    <conditionalFormat scope="data" priority="1">
+      <pivotAreas count="1">
+        <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+  </conditionalFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="0" type="count" evalOrder="-1" id="1" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="50" filterVal="50"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A4:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
@@ -23084,6 +23192,60 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="200" width="6.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mapa de calor: gasto por producto y mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué se mide: gasto mensual de cada producto, en € redondeados a la unidad (suma de lo pagado por ese producto en el mes). Filas: los 50 productos con más gasto en todo el periodo, de mayor a menor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Color: cuanto más rojo, más gasto ese mes, comparado con el resto de la tabla; en blanco, ese mes no se compró. Sirve para ver cambios de hábito (productos que desaparecen o que entran fuerte) y la estacionalidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Para ver más o menos productos: filtro de la fila → Filtros de valor → Diez mejores.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B9:B10" pivot="1">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FFFCC98F"/>
+        <color rgb="FFE0503C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D558"/>

</xml_diff>